<commit_message>
task FE-002 to FE-005 completetd
</commit_message>
<xml_diff>
--- a/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
+++ b/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
@@ -2409,11 +2409,23 @@
         <v>21</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="H3" s="5"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="5"/>
+        <v>519</v>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>aminullah-01</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Configured ESLint 9, Prettier, lint-staged, and Husky pre-commit hook. Verified pre-commit blocks lint failures and scripts pass.</t>
+        </is>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
@@ -2435,11 +2447,23 @@
         <v>15</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" s="5"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="5"/>
+        <v>519</v>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>aminullah-01</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Created .env.example and .env with VITE_API_BASE_URL and VITE_USE_MOCK_DATA switch. Verified .env is gitignored and src/utils/env.js works.</t>
+        </is>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
@@ -2461,11 +2485,23 @@
         <v>15</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="H5" s="5"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="5"/>
+        <v>519</v>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>aminullah-01</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Implemented React Router route map for all public, buyer, seller, admin and error routes matching SRS 4.1.2 with layout shells.</t>
+        </is>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
@@ -2487,11 +2523,23 @@
         <v>15</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="H6" s="5"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="5"/>
+        <v>519</v>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>aminullah-01</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Defined design tokens in src/utils/tokens.js and CSS custom properties in src/index.css for colours, typography, 8px spacing, and 360-1920px breakpoints.</t>
+        </is>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">

</xml_diff>

<commit_message>
task FE-006 to FE-010 completed
</commit_message>
<xml_diff>
--- a/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
+++ b/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
@@ -2300,7 +2300,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -2561,11 +2561,23 @@
         <v>15</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="H7" s="5"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="5"/>
+        <v>519</v>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>aminullah-01</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Implemented responsive layout shells (MainLayout with hamburger drawer, DashboardLayout with off-canvas sidebar), table-responsive wrappers, and 360-1920px overflow protections.</t>
+        </is>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
@@ -2587,11 +2599,23 @@
         <v>15</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="H8" s="5"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="5"/>
+        <v>519</v>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>aminullah-01</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Created formatters in src/utils/formatters.js: formatCurrency, formatPrice (₦2,500 / basket), formatDate/formatDateTime (Africa/Lagos WAT), and toUtcIso.</t>
+        </is>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
@@ -2613,7 +2637,7 @@
         <v>21</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H9" s="5"/>
       <c r="I9" s="7"/>
@@ -2639,7 +2663,7 @@
         <v>15</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H10" s="5"/>
       <c r="I10" s="7"/>
@@ -2665,7 +2689,7 @@
         <v>15</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H11" s="5"/>
       <c r="I11" s="7"/>
@@ -5703,7 +5727,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
+  <drawing ns1:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
task FE-011 to FE-015 implemented
</commit_message>
<xml_diff>
--- a/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
+++ b/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
@@ -2715,7 +2715,7 @@
         <v>15</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H12" s="5"/>
       <c r="I12" s="7"/>
@@ -2741,7 +2741,7 @@
         <v>15</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H13" s="5"/>
       <c r="I13" s="7"/>
@@ -2767,7 +2767,7 @@
         <v>15</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H14" s="5"/>
       <c r="I14" s="7"/>
@@ -2793,7 +2793,7 @@
         <v>15</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H15" s="5"/>
       <c r="I15" s="7"/>
@@ -2819,7 +2819,7 @@
         <v>15</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H16" s="5"/>
       <c r="I16" s="7"/>

</xml_diff>

<commit_message>
task FE-016 to FE-020 implemented
</commit_message>
<xml_diff>
--- a/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
+++ b/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
@@ -2845,7 +2845,7 @@
         <v>21</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H17" s="5"/>
       <c r="I17" s="7"/>
@@ -2871,7 +2871,7 @@
         <v>15</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H18" s="5"/>
       <c r="I18" s="7"/>
@@ -2897,7 +2897,7 @@
         <v>21</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H19" s="5"/>
       <c r="I19" s="7"/>
@@ -2923,7 +2923,7 @@
         <v>21</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H20" s="5"/>
       <c r="I20" s="7"/>
@@ -2949,7 +2949,7 @@
         <v>21</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H21" s="5"/>
       <c r="I21" s="7"/>

</xml_diff>

<commit_message>
task FE-020 to FE-025 completed
</commit_message>
<xml_diff>
--- a/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
+++ b/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
@@ -2974,8 +2974,8 @@
       <c r="F22" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G22" s="6" t="s">
-        <v>16</v>
+      <c r="G22" t="s">
+        <v>519</v>
       </c>
       <c r="H22" s="5"/>
       <c r="I22" s="7"/>
@@ -3000,8 +3000,8 @@
       <c r="F23" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G23" s="6" t="s">
-        <v>16</v>
+      <c r="G23" t="s">
+        <v>519</v>
       </c>
       <c r="H23" s="5"/>
       <c r="I23" s="7"/>
@@ -3027,7 +3027,7 @@
         <v>15</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H24" s="5"/>
       <c r="I24" s="7"/>
@@ -3053,7 +3053,7 @@
         <v>15</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H25" s="5"/>
       <c r="I25" s="7"/>
@@ -3079,7 +3079,7 @@
         <v>15</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H26" s="5"/>
       <c r="I26" s="7"/>

</xml_diff>

<commit_message>
task FE-26 to FE-30
</commit_message>
<xml_diff>
--- a/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
+++ b/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
@@ -3105,7 +3105,7 @@
         <v>15</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H27" s="5"/>
       <c r="I27" s="7"/>
@@ -3131,7 +3131,7 @@
         <v>15</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H28" s="5"/>
       <c r="I28" s="7"/>
@@ -3157,7 +3157,7 @@
         <v>21</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H29" s="5"/>
       <c r="I29" s="7"/>

</xml_diff>

<commit_message>
task 31 to 35 completed
</commit_message>
<xml_diff>
--- a/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
+++ b/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
@@ -3183,7 +3183,7 @@
         <v>15</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H30" s="5"/>
       <c r="I30" s="7"/>
@@ -3261,11 +3261,23 @@
         <v>21</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="H33" s="5"/>
-      <c r="I33" s="7"/>
-      <c r="J33" s="5"/>
+        <v>519</v>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>aminullah-01</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>Implemented SellerCard in src/components/products/SellerCard.jsx: business name, location, rating or "No ratings yet", short description and product count, plus a 44px "View Seller" link to /sellers/:id. Data-driven from seller_profiles columns and hides unapproved sellers from public listings (MKT-04). 14 tests added; lint, format, full suite and build pass.</t>
+        </is>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
@@ -3287,11 +3299,23 @@
         <v>15</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="H34" s="5"/>
-      <c r="I34" s="7"/>
-      <c r="J34" s="5"/>
+        <v>519</v>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>aminullah-01</t>
+        </is>
+      </c>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>Implemented shared SearchBar in src/components/common/SearchBar.jsx: keyword field with submit, trimmed/encoded into ?search= on /products (SRCH-01, SRCH-06), URL-synced input, optional clear action and 44px touch targets. Refactored Navbar desktop and mobile drawer to use it (removed duplicate inline forms) and added .search-bar styles. 16 tests added; lint, format, full suite (239 tests) and build pass.</t>
+        </is>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
@@ -3313,7 +3337,7 @@
         <v>15</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H35" s="5"/>
       <c r="I35" s="7"/>
@@ -3339,7 +3363,7 @@
         <v>15</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H36" s="5"/>
       <c r="I36" s="7"/>

</xml_diff>

<commit_message>
task FE-36 to FE-40 completed
</commit_message>
<xml_diff>
--- a/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
+++ b/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
@@ -3389,7 +3389,7 @@
         <v>15</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H37" s="5"/>
       <c r="I37" s="7"/>
@@ -3415,7 +3415,7 @@
         <v>15</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H38" s="5"/>
       <c r="I38" s="7"/>
@@ -3441,7 +3441,7 @@
         <v>15</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H39" s="5"/>
       <c r="I39" s="7"/>
@@ -3467,7 +3467,7 @@
         <v>15</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H40" s="5"/>
       <c r="I40" s="7"/>
@@ -3493,7 +3493,7 @@
         <v>175</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H41" s="5"/>
       <c r="I41" s="7"/>

</xml_diff>

<commit_message>
task FE-41 to FE-45 completed
</commit_message>
<xml_diff>
--- a/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
+++ b/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
@@ -3519,7 +3519,7 @@
         <v>15</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H42" s="5"/>
       <c r="I42" s="7"/>
@@ -3545,7 +3545,7 @@
         <v>15</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H43" s="5"/>
       <c r="I43" s="7"/>
@@ -3571,7 +3571,7 @@
         <v>15</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H44" s="5"/>
       <c r="I44" s="7"/>
@@ -3597,7 +3597,7 @@
         <v>21</v>
       </c>
       <c r="G45" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H45" s="5"/>
       <c r="I45" s="7"/>
@@ -3623,7 +3623,7 @@
         <v>15</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H46" s="5"/>
       <c r="I46" s="7"/>

</xml_diff>

<commit_message>
task FE-46 to FE-50 completed
</commit_message>
<xml_diff>
--- a/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
+++ b/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
@@ -3649,7 +3649,7 @@
         <v>15</v>
       </c>
       <c r="G47" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H47" s="5"/>
       <c r="I47" s="7"/>
@@ -3675,7 +3675,7 @@
         <v>15</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H48" s="5"/>
       <c r="I48" s="7"/>
@@ -3701,7 +3701,7 @@
         <v>15</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H49" s="5"/>
       <c r="I49" s="7"/>
@@ -3727,7 +3727,7 @@
         <v>15</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H50" s="5"/>
       <c r="I50" s="7"/>
@@ -3753,7 +3753,7 @@
         <v>15</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H51" s="5"/>
       <c r="I51" s="7"/>

</xml_diff>

<commit_message>
task FE-51 to FE-55 completed
</commit_message>
<xml_diff>
--- a/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
+++ b/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
@@ -3779,7 +3779,7 @@
         <v>15</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H52" s="5"/>
       <c r="I52" s="7"/>
@@ -3805,7 +3805,7 @@
         <v>21</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H53" s="5"/>
       <c r="I53" s="7"/>
@@ -3831,7 +3831,7 @@
         <v>21</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H54" s="5"/>
       <c r="I54" s="7"/>
@@ -3857,7 +3857,7 @@
         <v>15</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H55" s="5"/>
       <c r="I55" s="7"/>
@@ -3883,7 +3883,7 @@
         <v>15</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H56" s="5"/>
       <c r="I56" s="7"/>

</xml_diff>

<commit_message>
task FE-56 to FE-60 completed
</commit_message>
<xml_diff>
--- a/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
+++ b/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
@@ -3909,7 +3909,7 @@
         <v>15</v>
       </c>
       <c r="G57" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H57" s="5"/>
       <c r="I57" s="7"/>
@@ -3935,7 +3935,7 @@
         <v>15</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H58" s="5"/>
       <c r="I58" s="7"/>
@@ -3961,7 +3961,7 @@
         <v>21</v>
       </c>
       <c r="G59" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H59" s="5"/>
       <c r="I59" s="7"/>
@@ -3987,7 +3987,7 @@
         <v>15</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H60" s="5"/>
       <c r="I60" s="7"/>
@@ -4013,7 +4013,7 @@
         <v>15</v>
       </c>
       <c r="G61" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H61" s="5"/>
       <c r="I61" s="7"/>

</xml_diff>

<commit_message>
task FE-61 to FE-62 completed
</commit_message>
<xml_diff>
--- a/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
+++ b/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
@@ -4039,7 +4039,7 @@
         <v>175</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H62" s="5"/>
       <c r="I62" s="7"/>
@@ -4065,7 +4065,7 @@
         <v>15</v>
       </c>
       <c r="G63" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H63" s="5"/>
       <c r="I63" s="7"/>

</xml_diff>

<commit_message>
feat(testing): implement task FE-112 unit tests for cart, validation, and utilities (NFR-MAIN-04)
</commit_message>
<xml_diff>
--- a/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
+++ b/Vegetable-joint-all-document/Vegetable_Joint_Frontend_Tasks.xlsx
@@ -2300,7 +2300,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -5365,7 +5365,7 @@
         <v>21</v>
       </c>
       <c r="G113" s="6" t="s">
-        <v>16</v>
+        <v>519</v>
       </c>
       <c r="H113" s="5"/>
       <c r="I113" s="7"/>
@@ -5751,7 +5751,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
+  <drawing ns1:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>